<commit_message>
S03-S10: add persistent core workflows
</commit_message>
<xml_diff>
--- a/fixtures/northstar/Northstar_Diligence_Tracker.xlsx
+++ b/fixtures/northstar/Northstar_Diligence_Tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="35">
   <si>
     <t>ID</t>
   </si>
@@ -19,16 +19,55 @@
     <t>Request</t>
   </si>
   <si>
-    <t>Contracts</t>
-  </si>
-  <si>
-    <t>FY25 revenue</t>
-  </si>
-  <si>
-    <t>FY26 revenue</t>
-  </si>
-  <si>
-    <t>Expiry dates</t>
+    <t>Workstream</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Requested from</t>
+  </si>
+  <si>
+    <t>Approved status</t>
+  </si>
+  <si>
+    <t>Due</t>
+  </si>
+  <si>
+    <t>Coverage</t>
+  </si>
+  <si>
+    <t>F-02</t>
+  </si>
+  <si>
+    <t>Monthly management accounts</t>
+  </si>
+  <si>
+    <t>Prepared</t>
+  </si>
+  <si>
+    <t>Awaiting response</t>
+  </si>
+  <si>
+    <t>No response received</t>
+  </si>
+  <si>
+    <t>F-05</t>
+  </si>
+  <si>
+    <t>Quality of earnings bridge</t>
+  </si>
+  <si>
+    <t>C-03</t>
+  </si>
+  <si>
+    <t>Customer churn cohorts</t>
+  </si>
+  <si>
+    <t>C-08</t>
+  </si>
+  <si>
+    <t>Sales pipeline and conversion</t>
   </si>
   <si>
     <t>C-14</t>
@@ -37,7 +76,46 @@
     <t>Customer concentration information</t>
   </si>
   <si>
-    <t>Required</t>
+    <t>T-04</t>
+  </si>
+  <si>
+    <t>Platform architecture overview</t>
+  </si>
+  <si>
+    <t>T-09</t>
+  </si>
+  <si>
+    <t>Security incident history</t>
+  </si>
+  <si>
+    <t>L-02</t>
+  </si>
+  <si>
+    <t>Material customer agreements</t>
+  </si>
+  <si>
+    <t>L-06</t>
+  </si>
+  <si>
+    <t>Open litigation and disputes</t>
+  </si>
+  <si>
+    <t>P-03</t>
+  </si>
+  <si>
+    <t>Leadership employment terms</t>
+  </si>
+  <si>
+    <t>P-07</t>
+  </si>
+  <si>
+    <t>Employee attrition analysis</t>
+  </si>
+  <si>
+    <t>I-01</t>
+  </si>
+  <si>
+    <t>Insurance policies and claims</t>
   </si>
 </sst>
 </file>
@@ -414,10 +492,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -436,25 +514,237 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
-        <v>8</v>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" t="s">
+        <v>11</v>
+      </c>
+      <c r="H18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" t="s">
+        <v>11</v>
+      </c>
+      <c r="H23" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>26</v>
+      </c>
+      <c r="C26" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" t="s">
+        <v>11</v>
+      </c>
+      <c r="H26" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" t="s">
+        <v>10</v>
+      </c>
+      <c r="F30" t="s">
+        <v>11</v>
+      </c>
+      <c r="H30" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" t="s">
+        <v>10</v>
+      </c>
+      <c r="F32" t="s">
+        <v>11</v>
+      </c>
+      <c r="H32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" t="s">
+        <v>32</v>
+      </c>
+      <c r="C34" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" t="s">
+        <v>11</v>
+      </c>
+      <c r="H34" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>33</v>
+      </c>
+      <c r="B35" t="s">
+        <v>34</v>
+      </c>
+      <c r="C35" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" t="s">
+        <v>11</v>
+      </c>
+      <c r="H35" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S03-S10: add persistent core workflows (#2)
</commit_message>
<xml_diff>
--- a/fixtures/northstar/Northstar_Diligence_Tracker.xlsx
+++ b/fixtures/northstar/Northstar_Diligence_Tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="35">
   <si>
     <t>ID</t>
   </si>
@@ -19,16 +19,55 @@
     <t>Request</t>
   </si>
   <si>
-    <t>Contracts</t>
-  </si>
-  <si>
-    <t>FY25 revenue</t>
-  </si>
-  <si>
-    <t>FY26 revenue</t>
-  </si>
-  <si>
-    <t>Expiry dates</t>
+    <t>Workstream</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Requested from</t>
+  </si>
+  <si>
+    <t>Approved status</t>
+  </si>
+  <si>
+    <t>Due</t>
+  </si>
+  <si>
+    <t>Coverage</t>
+  </si>
+  <si>
+    <t>F-02</t>
+  </si>
+  <si>
+    <t>Monthly management accounts</t>
+  </si>
+  <si>
+    <t>Prepared</t>
+  </si>
+  <si>
+    <t>Awaiting response</t>
+  </si>
+  <si>
+    <t>No response received</t>
+  </si>
+  <si>
+    <t>F-05</t>
+  </si>
+  <si>
+    <t>Quality of earnings bridge</t>
+  </si>
+  <si>
+    <t>C-03</t>
+  </si>
+  <si>
+    <t>Customer churn cohorts</t>
+  </si>
+  <si>
+    <t>C-08</t>
+  </si>
+  <si>
+    <t>Sales pipeline and conversion</t>
   </si>
   <si>
     <t>C-14</t>
@@ -37,7 +76,46 @@
     <t>Customer concentration information</t>
   </si>
   <si>
-    <t>Required</t>
+    <t>T-04</t>
+  </si>
+  <si>
+    <t>Platform architecture overview</t>
+  </si>
+  <si>
+    <t>T-09</t>
+  </si>
+  <si>
+    <t>Security incident history</t>
+  </si>
+  <si>
+    <t>L-02</t>
+  </si>
+  <si>
+    <t>Material customer agreements</t>
+  </si>
+  <si>
+    <t>L-06</t>
+  </si>
+  <si>
+    <t>Open litigation and disputes</t>
+  </si>
+  <si>
+    <t>P-03</t>
+  </si>
+  <si>
+    <t>Leadership employment terms</t>
+  </si>
+  <si>
+    <t>P-07</t>
+  </si>
+  <si>
+    <t>Employee attrition analysis</t>
+  </si>
+  <si>
+    <t>I-01</t>
+  </si>
+  <si>
+    <t>Insurance policies and claims</t>
   </si>
 </sst>
 </file>
@@ -414,10 +492,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -436,25 +514,237 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
-        <v>8</v>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" t="s">
+        <v>11</v>
+      </c>
+      <c r="H18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" t="s">
+        <v>11</v>
+      </c>
+      <c r="H23" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>26</v>
+      </c>
+      <c r="C26" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" t="s">
+        <v>11</v>
+      </c>
+      <c r="H26" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" t="s">
+        <v>10</v>
+      </c>
+      <c r="F30" t="s">
+        <v>11</v>
+      </c>
+      <c r="H30" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" t="s">
+        <v>10</v>
+      </c>
+      <c r="F32" t="s">
+        <v>11</v>
+      </c>
+      <c r="H32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" t="s">
+        <v>32</v>
+      </c>
+      <c r="C34" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" t="s">
+        <v>11</v>
+      </c>
+      <c r="H34" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>33</v>
+      </c>
+      <c r="B35" t="s">
+        <v>34</v>
+      </c>
+      <c r="C35" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" t="s">
+        <v>11</v>
+      </c>
+      <c r="H35" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>